<commit_message>
update cohort summary results
</commit_message>
<xml_diff>
--- a/CPRD Raw Analysis/Results/cohort_summary_raw.xlsx
+++ b/CPRD Raw Analysis/Results/cohort_summary_raw.xlsx
@@ -385,6 +385,18 @@
       <c r="A2">
         <v>25138</v>
       </c>
+      <c r="B2">
+        <v>517</v>
+      </c>
+      <c r="C2">
+        <v>2.06</v>
+      </c>
+      <c r="D2">
+        <v>24621</v>
+      </c>
+      <c r="E2">
+        <v>97.94</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>